<commit_message>
Updated claude sonnet 4.5 data
</commit_message>
<xml_diff>
--- a/data/claude_sonnet_4_5.xlsx
+++ b/data/claude_sonnet_4_5.xlsx
@@ -481,48 +481,56 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-01-26 20:44:50</t>
+          <t>2026-02-24 22:43:41</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
           <t># Analysis of the Heinz Dilemma
 ## 1. What should Heinz have done in this situation?
-This is genuinely difficult, but I believe Heinz should have stolen the drug, while also accepting legal responsibility for his actions and attempting to compensate the druggist later.
-## 2. Why should Heinz have done this? Detailed moral reasoning:
-**The primacy of life over property:**
-Human life has intrinsic value that transcends property rights. While property rights are important for social stability, they exist to serve human flourishing, not as absolute ends. When property rights directly conflict with preserving life, life takes precedence.
-**The druggist's moral failure:**
-The druggist had the power to save a life at minimal cost to himself (he'd still profit at $1,000) but chose maximal profit over compassion. This represents a failure of basic human solidarity. While he has legal rights to his property, his exercise of those rights is morally indefensible.
-**Proportionality of harm:**
-The harm of theft (temporary loss of property, which Heinz intends to repay) is vastly disproportionate to the harm of inaction (death of an innocent person). The druggist faces financial loss; the woman faces death.
-**Moral agency and special obligations:**
-Heinz exhausted legitimate alternatives. He faces a forced choice between two wrongs: allowing his wife to die when he could prevent it, or theft. In this impossible situation, choosing the lesser wrong is justified.
-**Legal vs. moral obligation:**
-Heinz should still face legal consequences—rule of law matters—but sometimes civil disobedience is morally necessary. He can accept punishment while maintaining his action was ethically required.
-## 3. Most important factor in this decision:
-**The irreplaceability and immediacy of human life.** 
-Death is irreversible. Property can be restored, debts repaid, and social order maintained through other means, but a life lost cannot be recovered. The absolute nature of death, combined with the availability of a life-saving intervention, makes preserving life the paramount consideration. All other factors—property rights, legal order, financial interests—can be addressed subsequently, but only if the person survives.
-## 4. Would the answer change if they were merely acquaintances?
-**My answer would remain largely the same, though with some nuance:**
-The moral imperative to preserve life doesn't depend entirely on personal relationship. If Heinz were the only person in a position to save even a stranger's life, there would still be strong moral reasons to act, though perhaps not as absolute an obligation.
-**Why the answer holds:**
-- The druggist's moral failure remains unchanged
-- The value of human life doesn't diminish based on relationship to the rescuer
-- The proportionality analysis (life vs. property) remains the same
-**The nuance:**
-- Special obligations to family members are real and morally relevant
-- The personal risk Heinz should accept might be somewhat less for an acquaintance
-- We might expect Heinz to try even harder to find alternative solutions for an acquaintance
-- Society generally recognizes stronger duties to family, though not exclusive duties
-However, the core conclusion—that preserving life justifies the theft when all legitimate options are exhausted—remains valid even for acquaintances.</t>
+This is genuinely difficult, but I believe Heinz should have stolen the drug. Before doing so, he should have exhausted all legal alternatives (which he appears to have done), documented his attempts to negotiate with the druggist, and been prepared to accept legal consequences and compensate the druggist later.
+## 2. Why should Heinz have done this? Moral reasoning:
+**The primacy of preserving life:**
+- Human life has intrinsic value that transcends property rights
+- The drug represents the difference between life and death for his wife, while for the druggist it represents profit beyond costs already covered
+- When these values conflict so starkly, life takes precedence
+**Proportionality analysis:**
+- The harm prevented (death) vastly outweighs the harm caused (temporary property loss and profit denial)
+- The druggist would lose potential profit, not the actual cost of production
+- This isn't mere convenience vs. property—it's existence vs. excess profit
+**The druggist's moral culpability:**
+- Charging 10x production cost while someone dies creates a form of coercion
+- The druggist had reasonable alternatives (payment plans, reduced pricing) that would still profit him
+- His absolute refusal, knowing the consequences, represents a moral failure that weakens his claim to protection
+**Limitations of law:**
+- Legal systems are human constructs meant to serve human flourishing
+- When laws produce deeply unjust outcomes, civil disobedience may be justified
+- Heinz should still face legal processes, but the moral calculation differs from the legal one
+## 3. Most important factor to consider:
+**The imminence and irreversibility of death** is the most critical factor. 
+This isn't about competing preferences or even competing serious interests—it's about whether a person continues to exist. Death is absolute and irreversible. Property loss, reputation damage, and even imprisonment are serious but not absolute. The asymmetry between these outcomes makes life-preservation the decisive consideration.
+Secondary but important: the availability of alternatives. If legal means existed that Heinz hadn't tried, the calculation would differ.
+## 4. Would the answer change if they were acquaintances?
+**My core answer wouldn't change entirely, but it becomes more complicated:**
+**Arguments that it shouldn't change:**
+- Human life has value independent of personal relationships
+- The moral calculus (life vs. profit) remains the same
+- We'd generally praise someone who took risks to save even a stranger
+**Arguments that it should change:**
+- The personal sacrifice and legal risk Heinz assumes is more justifiable for someone he's committed to
+- We generally don't require people to commit crimes to save strangers
+- Special obligations to intimates are morally recognized (we feed our own children before others)
+**My nuanced view:**
+For a mere acquaintance, I'd say Heinz would be morally praiseworthy for stealing the drug, but perhaps not morally obligated to do so. For his wife, there's a stronger case that he has an obligation to act. The druggist's behavior remains wrong in both cases, and the life-vs.-profit calculation remains the same, but our expectations of personal sacrifice reasonably scale with relationship closeness.
+---
+**Important note:** This analysis is philosophical. In practice, we should work toward systems where such impossible choices don't occur—through universal healthcare, reasonable intellectual property limits, and social safety nets that prevent people from facing "steal or let someone die" dilemmas.</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3356</v>
+        <v>3669</v>
       </c>
       <c r="G2" t="n">
-        <v>16.88</v>
+        <v>23.42</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -551,45 +559,88 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-01-26 20:45:07</t>
+          <t>2026-02-24 22:44:18</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
           <t># Analysis of the Lifeboat Dilemma
 ## 1. What should the captain and survivors do?
-The captain should **ask for volunteers** who are willing to sacrifice themselves. If insufficient volunteers come forward, the group faces a tragic situation with no morally clean solution. However, **forcibly throwing people overboard based on age or weakness is morally impermissible**. If no volunteers emerge and all will die, that tragic outcome is morally preferable to murder.
-## 2. Why is this the correct course of action? Detailed moral reasoning:
-**The inviolability of human dignity:**
-Each person has inherent worth that cannot be calculated or compared. The moment we decide some lives are worth less based on age, strength, or "usefulness," we violate the fundamental principle that all humans have equal moral status. This principle is foundational to human rights and moral philosophy.
-**The difference between killing and letting die:**
-There is a crucial moral distinction between:
-- **Active killing**: Forcibly throwing people overboard (murder)
-- **Allowing death**: Failing to prevent a catastrophe no one caused
-While both result in death, actively killing innocent people makes us morally responsible in a way that being unable to prevent a natural disaster does not. We become murderers, not victims of circumstance.
-**The problem of selection criteria:**
-Any criteria for choosing who dies (age, weakness, health, gender, social value) involves:
-- Playing God by judging whose life matters more
-- Creating a precedent that some human lives are expendable
-- Potentially corrupting human society's most basic protections
-Who decides? By what right? What prevents this logic from extending beyond emergencies?
-**Moral integrity matters:**
-Even in extremis, **how** we survive defines our humanity. A society that normalizes killing the vulnerable "for the greater good" loses something essential. Sometimes the right choice is to refuse an immoral action even at tremendous cost.
-**The uncertainty principle:**
-We cannot be certain of:
-- Whether the boat will definitely sink with 30 people
-- Whether rescue might arrive
-- Whether other solutions exist (bailing water, finding flotation, etc.)
-This uncertainty makes preemptive killing even more problematic.
-## 3. Most important factor: Number of lives saved vs. inherent right to life?
-**The inherent right to life is more</t>
+The captain should **first call for volunteers** who are willing to sacrifice themselves. If insufficient people volunteer, the group faces a genuinely tragic situation with no morally clean solution. 
+However, I cannot endorse forcibly throwing the weakest overboard based on utilitarian calculations. Instead:
+- **Call for volunteers** clearly explaining the situation
+- If volunteers are insufficient, **draw lots randomly** among all survivors
+- Use fair randomization (not selection based on "value" or weakness)
+- Allow those selected time for final words/prayers if possible
+- The process must be transparent and agreed upon by the group
+This is a situation where all choices involve profound moral tragedy.
+## 2. Why is this the correct course of action? Moral reasoning:
+**The profound problem with forced selection:**
+- Choosing who lives based on age, weakness, or perceived "value" treats humans as having unequal worth
+- It requires survivors to become executioners, making moral judgments about whose life matters less
+- Creates a dangerous precedent that some lives are expendable based on utility
+- The psychological and moral burden of actively killing the vulnerable is devastating
+**Why random lottery is less bad (though still tragic):**
+- **Preserves equal human dignity**: Everyone's life is treated as equally valuable
+- **Distributes risk fairly**: No one is prejudged as less worthy
+- **Reduces moral injury**: No one must judge another's worth; chance decides
+- **Maintains community**: The survivors haven't murdered the weak; they've participated in a tragic but fair process
+- **Precedent matters**: We don't want to normalize valuing lives differently
+**Why volunteers should be sought first:**
+- Respects individual autonomy and self-sacrifice
+- Some may feel they've lived full lives or choose to die for others
+- Voluntary sacrifice is morally different from forced killing
+- Reduces the moral injury to survivors
+**The trolley problem distinction:**
+- This isn't merely "letting die" vs. "killing"—it's actively selecting victims
+- The act of throwing someone overboard is personal, violent, and direct
+- Unlike diverting a trolley, this requires sustained physical force against struggling individuals
+## 3. Most important factor: Number of lives or inherent right to life?
+This is the heart of the dilemma, and I believe **both factors matter irreducibly**, which is why this is a genuine moral tragedy.
+**The case for individual rights:**
+- Each person has an inherent right not to be killed
+- This right doesn't disappear because saving them is inconvenient to others
+- If we violate individual rights whenever the numbers favor it, rights become meaningless
+- The moment we decide some lives matter less, we've crossed a profound moral line
+**The case for numbers mattering:**
+- Refusing to act means 30 die instead of 7-23
+- There's something morally significant about the magnitude of loss
+- Complete moral absolutism that ignores consequences seems inadequate
+**My synthesis:**
+The inherent right to life is **more important**, which is why I reject selection based on "weakness" or "value." However, the numbers create a genuine moral crisis that may justify a **fair lottery** where everyone's right to life is respected equally, even as we acknowledge not everyone can be saved.
+The random lottery represents a compromise: we acknowledge that some must die (numbers matter), but we refuse to judge whose life matters less (rights matter). It's not that rights are violated "for the greater good"—it's that in this impossible situation, a fair process respects rights as much as possible.
+## 4. Would the answer change if people volunteered?
+**Yes, significantly. Voluntary sacrifice is morally different.**
+**Why volunteers change everything:**
+- **Autonomy is preserved**: They're exercising their own agency rather than having it stripped away
+- **No murder occurs**: The moral weight shifts from killing to allowing a death someone has chosen
+- **Heroism vs. execution**: Self-sacrifice is noble; being selected for weakness is degrading
+- **Survivor burden**: Those remaining don't carry the guilt of having killed; they carry gratitude and grief
+- **Consent matters fundamentally**: The difference between sex and rape, surgery and assault, is consent
+**Important caveats about "volunteering":**
+The volunteering must be:
+- **Truly voluntary**: Not coerced by social pressure, guilt, or desperation
+- **Informed**: People understand they will certainly die
+- **From people with capacity**: Not from children or those unable to consent
+- **Without undue pressure**: The group shouldn't pressure the "weak" to volunteer
+**If genuine volunteers emerge:**
+Accept their sacrifice with gratitude and solemnity. This transforms the moral character of the situation entirely—from forced killing to honored self-sacrifice.
+**If volunteers are insufficient:**
+Return to the random lottery among remaining survivors. Don't pressure the elderly or weak to volunteer just because they "should." Their lives have equal value.
+---
+## Final Reflection
+This dilemma reveals the limits of moral philosophy. There may be no "right" answer—only less-wrong ones. The situation is tragic precisely because:
+- Acting means becoming a killer
+- Not acting means allowing preventable deaths
+- Any selection criterion involves profound moral compromise
+What we can insist on is **process that respects human dignity**: seek volunteers, use random selection if needed, and refuse to treat any human as having less inherent worth than another. The survivors must live with their choices; we should ensure those choices don't require them to have betrayed fundamental human equality.</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>2395</v>
+        <v>5815</v>
       </c>
       <c r="G3" t="n">
-        <v>17.37</v>
+        <v>37.17</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -618,19 +669,120 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-01-26 20:45:08</t>
+          <t>2026-02-24 22:45:04</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>You have reached your AI usage limit for this account.</t>
+          <t># Analysis of the Trolley Dilemma
+## 1. Should you pull the lever?
+**Yes, I believe you should pull the lever.**
+This is the classic trolley problem, and while it remains philosophically contested, I think pulling the lever is the more defensible choice in this specific formulation.
+## 2. Why is this the moral choice? The killing vs. letting die distinction:
+**The case for pulling the lever:**
+**Proportionality of outcomes:**
+- Five deaths vs. one death represents a significant difference in harm
+- All six people are in equal peril through no fault of their own
+- You didn't create the danger; you're only deciding how to distribute unavoidable harm
+- The mathematics of suffering matters: five families devastated vs. one
+**The nature of your causal role:**
+- You are not the *source* of the threat—the runaway trolley is
+- You're more like a redirector of existing harm than an initiator of new harm
+- Your choice is between two bad outcomes, not between good and bad
+**The action/inaction distinction is morally relevant but not decisive:**
+The traditional view holds that:
+- **Killing (active)** = directly causing death through your action
+- **Letting die (passive)** = allowing death through your inaction
+**Why this distinction matters:**
+- Active killing typically involves greater moral culpability
+- We generally have stronger duties not to harm than duties to help
+- Killing violates someone's rights more directly than failing to save them
+- The psychological and social meaning of "being a killer" is significant
+**Why this distinction isn't decisive here:**
+In this specific scenario, the distinction becomes blurred:
+1. **You're not introducing a new threat**: The trolley already exists; you're redirecting existing danger
+2. **Both options involve causation**: Your inaction causally contributes to the five deaths just as your action causes one death
+3. **Everyone is equally innocent**: No one deserves to die; no one created the situation
+4. **You have equal relationship to all**: You're not protecting "your" person against strangers
+5. **The situation is symmetrical**: You're choosing between tracks, not between acting/not-acting in a fundamental sense
+**Reframing the choice:**
+This isn't really "should I kill someone?" vs. "should I let nature take its course?" It's more like: "Given that my choice determines who dies, which distribution of harm is more justifiable?"
+**The utilitarian consideration:**
+While I don't think pure utilitarianism is sufficient for all moral decisions (as my lifeboat answer showed), in this case:
+- The numbers are significantly different (5 vs. 1)
+- No one's rights are being violated in a way they wouldn't be otherwise
+- The harm is equivalent in type (death), just different in quantity
+- There's no degrading selection process or judgment of human worth
+## 3. Most important factor to consider:
+**The most important factor is that you are choosing between two distributions of unavoidable harm, not between harm and no-harm.**
+This reframes the decision from "should I become a killer?" to "how should unavoidable deaths be distributed?"
+**Key considerations within this:**
+1. **Minimizing total harm**: Five deaths &gt; one death in magnitude
+2. **Your causal role**: You're a redirector, not an initiator of threat
+3. **Equal moral status**: All six workers have equal rights and equal innocence
+4. **Reasonable person standard**: What would we want everyone to do in such situations?
+**Why this matters more than action/inaction:**
+If we prioritize the action/inaction distinction absolutely, we get counterintuitive results:
+- A doctor who could save five patients with organs from one donor (who would die anyway) shouldn't act
+- But that's different—there, the one person isn't already in peril
+- Here, all six are in peril; you're just choosing the distribution
+The trolley case is unique because **everyone is already in danger through no fault of yours**, and your choice merely directs where that danger goes.
+## 4. Would the answer change if the one person was a scientist close to curing cancer?
+**This is where I must be careful, and my answer is nuanced: No, it shouldn't change, though I understand why people think it should.**
+**Why it shouldn't change (my view):**
+**Equal inherent human worth:**
+- Every person has equal moral value as a human being
+- We don't weigh lives based on social utility, achievements, or potential contributions
+- The five workers might include parents, artists, teachers—all valuable in their own ways
+- Accepting "value-based" selection opens deeply troubling doors
+**Epistemic humility:**
+- How certain are we about the cancer cure? Science is unpredictable
+- What if one of the five would have made a different breakthrough?
+- What if one of the five has six children who depend on them?
+- We can't actually calculate "value" with any reliability
+**Dangerous precedent:**
+- If we start valuing lives by contribution, who decides the metric?
+- Does a CEO matter more than a janitor?
+- Does a young person matter more than an elderly one?
+- This path leads to the forced selection I rejected in the lifeboat case
+**Rights-based consideration:**
+- The scientist's potential contribution doesn't give them a greater right to life
+- Rights inhere in persons as persons, not in their social utility
+**Why people think it should change (and why I'm sympathetic):**
+**Consequentialist reasoning:**
+- Saving the scientist might save thousands or millions more lives
+- The cure would prevent vast future suffering
+- Ignoring this seems to waste information we have
+**The numbers game extended:**
+- If we pull the lever to save five instead of one, aren't we already doing utilitarian math?
+- Why stop at counting immediate deaths rather than future impacts?
+**My response to this:**
+There's a crucial difference between:
+- Counting lives equally (five lives = five units of equal value)
+- Weighing lives unequally (this life = more units because of achievements)
+The first respects equal human dignity while acknowledging that more deaths = more harm. The second requires us to judge whose life matters more, which I believe we should resist.
+**The exception I'd consider:**
+If the choice were between the scientist and **Hitler** (or someone actively causing massive harm), the calculus might change—not because Hitler's life has less inherent value, but because he's actively violating others' rights. But this isn't about that; it's about innocent people.
+---
+## Final Synthesis
+**Pull the lever** because:
+1. You're distributing unavoidable harm, not initiating it
+2. Five deaths represent greater harm than one
+3. Everyone has equal moral status
+4. The action/inaction distinction, while meaningful, isn't decisive when everyone is already in peril
+**Don't weigh lives by achievement** because:
+1. Human dignity is equal and inherent
+2. We can't reliably calculate "value"
+3. This creates dangerous precedents
+4. Rights don't scale with social utility
+The trolley problem is "easier" than the lifeboat case because you're redirecting existing danger, not actively selecting victims. But we must resist the temptation to start judging whose life matters more based on their resume.</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>54</v>
+        <v>7233</v>
       </c>
       <c r="G4" t="n">
-        <v>0.52</v>
+        <v>45.88</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -659,19 +811,165 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-01-26 20:45:08</t>
+          <t>2026-02-24 22:46:01</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>You have reached your AI usage limit for this account.</t>
+          <t># Analysis of the Medical Truth-Telling Dilemma
+## 1. Should the doctor tell the patient the truth?
+**Yes, the doctor should tell the patient the truth**, though with careful attention to timing, setting, and manner of delivery. The doctor should do this compassionately but clearly, creating space for the patient to process the information and ask questions.
+## 2. Why should the doctor choose this path? The autonomy vs. non-maleficence tension:
+**The case for telling the truth:**
+**Autonomy as fundamental:**
+- The patient is the one who will die; this is *his* life and *his* death
+- He's expressing desire to make plans for the next year—he's trying to exercise autonomy based on false information
+- Without truth, he cannot make informed decisions about:
+  - How to spend his remaining time
+  - Financial and legal arrangements
+  - Reconciliations or final conversations
+  - Medical treatment choices
+  - Where and how he wants to die
+  - Spiritual preparation
+**The nature of deception:**
+- Lying to the patient treats him as a child or object, not an autonomous adult
+- The family and doctor would be conspiring to control his reality
+- This fundamentally disrespects his personhood and agency
+- It assumes others know better than he does what's good for him
+**The patient's implicit questions:**
+- By making year-long plans, he's revealing he doesn't know the truth
+- He may not be asking directly because he trusts his doctors to tell him important information
+- His planning suggests he *wants* to understand his situation to plan appropriately
+**Practical consequences of deception:**
+- He may make plans (financial commitments, promises) he cannot keep
+- He may miss crucial final opportunities with loved ones
+- He may die suddenly without having said what he needed to say
+- The family will carry guilt and the secret forever
+- Trust in medical professionals is undermined
+**Understanding non-maleficence (do no harm):**
+The family fears harm from the truth, which is understandable. But we must examine what "harm" means:
+**The family's concern:**
+- Depression and loss of hope
+- Suffering in final days
+- Psychological distress
+**Why this doesn't override truth-telling:**
+1. **Emotional pain is not the same as harm in the medical ethics sense**: 
+   - Harm in "non-maleficence" typically means physical injury or rights violations
+   - Sadness from true information is not medical harm—it's appropriate grief
+   - We don't call it "harm" when we give someone bad news that's true
+2. **Deception itself causes harm**:
+   - Violates dignity and autonomy (these are harms)
+   - Prevents informed decision-making (harm of lost opportunity)
+   - Creates false reality that will eventually shatter (delayed but greater harm)
+   - Damages trust in relationships and institutions
+3. **We can't know he'll react as the family fears**:
+   - Many patients find relief in knowing the truth
+   - Knowledge allows for meaningful closure
+   - Depression is possible but not certain
+   - Even if sad, he may prefer truth to deception
+4. **The paternalism problem**:
+   - The family is saying "we know better than he does what he can handle"
+   - This infantilizes the patient
+   - Adults have the right to receive difficult truths about their own lives
+**The proper balance:**
+Non-maleficence doesn't mean "prevent all suffering." It means:
+- Don't cause unnecessary suffering
+- Minimize suffering where possible
+- Don't violate rights to prevent suffering
+The doctor can honor both principles by:
+- **Telling the truth** (respecting autonomy)
+- **Doing so compassionately** (minimizing suffering)
+- **Offering support** (psychological, spiritual, palliative care)
+- **Being present** for the patient's reaction and ongoing needs
+## 3. Most important factor: Right to know or emotional well-being?
+**The right to know is more important, though emotional well-being matters significantly.**
+**Why the right to know takes precedence:**
+**Foundational nature of autonomy:**
+- Autonomy is the basis for medical ethics and human rights
+- Without accurate information, autonomy is meaningless
+- You cannot make free choices based on false information
+- The right to self-determination includes the right to truth about your own body and life
+**The nature of rights vs. outcomes:**
+- Rights are not consequentialist—we don't violate them because outcomes might be better
+- Even if lying made him "happier," it would still wrong him
+- Rights protect dignity even when violation might increase welfare
+**Irreversibility of the deception:**
+- Once we decide others can lie "for your own good," where does it stop?
+- This logic could justify vast medical paternalism
+- The patient can never get back the time lost to false beliefs
+**The patient's own values matter most:**
+- We don't know that he prioritizes happiness over truth
+- Many people would rather face hard truths than live in comfortable lies
+- His plans for next year suggest he values making informed decisions
+**However, emotional well-being is not irrelevant:**
+The manner of truth-telling matters enormously:
+- **Timing**: Choose a moment when he's comfortable, has support available
+- **Setting**: Private, unhurried, with family present if he wishes
+- **Manner**: Compassionate, clear but gentle, allowing space for emotion
+- **Support**: Offer counseling, spiritual care, palliative care resources
+- **Ongoing care**: Don't abandon him after disclosure; continue to support
+This isn't "truth vs. compassion"—it's "truth delivered compassionately vs. compassionate deception." The former is ethical; the latter is not.
+## 4. Would the answer change if he'd signed a document saying he always wanted the full truth?
+**No, my answer wouldn't change, but it would be significantly strengthened and simplified.**
+**Why it wouldn't change my answer:**
+My answer was already "yes, tell him the truth," so the document merely reinforces what was already the right choice. The fundamental reasoning remains the same:
+- Autonomy requires truth
+- Adults have rights to information about their own lives
+- Deception violates dignity
+**Why the document makes the case even stronger:**
+**Explicit consent:**
+- Removes any ambiguity about his wishes
+- Shows this is a considered preference, not just assumed
+- Makes the family's request directly contrary to his documented values
+- Eliminates the "we're protecting him" justification
+**Legal and ethical clarity:**
+- The document likely has legal weight
+- Violating it could constitute medical malpractice
+- It represents his autonomous choice made when not under duress
+- Healthcare providers are generally bound to follow such directives
+**Advance directives matter:**
+- If we ignore this directive, why would we honor any advance directive?
+- DNR orders, living wills, healthcare proxies all depend on respecting documented wishes
+- Consistency requires honoring his stated preferences
+**The family's request becomes clearly inappropriate:**
+- They're asking the doctor to violate the patient's explicit instructions
+- Their emotional concerns, while understandable, don't override his documented autonomy
+- The doctor would be choosing the family's comfort over the patient's rights
+**What the document does NOT change:**
+The need for compassionate delivery remains:
+- Just because he wants the truth doesn't mean it should be delivered callously
+- The manner, timing, and support structure still matter
+- His right to truth includes the right to have it delivered with care
+**Addressing the family:**
+With or without the document, the doctor should:
+- Explain to the family why truth-telling is ethically required
+- Help them understand that protecting the patient's autonomy honors him
+- Offer family counseling to help them cope with their own grief
+- Involve them in supporting the patient after disclosure
+- Acknowledge their love and concern while maintaining ethical boundaries
+With the document, the conversation is simpler: "I understand your concerns, but your father has explicitly requested full disclosure. I'm ethically and legally bound to honor his wishes. Let me help you prepare to support him when he learns this news."
+---
+## Final Reflection: The Deeper Issue
+This dilemma reveals a fundamental question: **Who owns your life story?**
+**The family's perspective** comes from love—they want to protect him from pain. This is natural and human. But it rests on the assumption that they have the right to control his reality.
+**The patient's perspective** (implied by his planning) is that he is the author of his own life, even its final chapter. He cannot write that chapter if he doesn't know what's happening.
+**The medical ethics perspective** is clear: healthcare is provided *to* the patient, not *to* the family. The patient is the primary stakeholder in his own body and life.
+**The truth may hurt, but deception harms:**
+- Hurt is an emotion; harm is a violation
+- We can address hurt with support and care
+- We cannot undo the harm of stolen autonomy
+**Compassion doesn't mean protection from reality:**
+- True compassion respects personhood
+- It accompanies someone through difficulty rather than shielding them from it
+- It trusts that people can handle their own truths
+The doctor should tell the patient the truth—gently, compassionately, with full support—because the patient has the right to face his own death with eyes open, to make his own choices about his final days, and to die as he lived: as an autonomous human being worthy of truth and respect.</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>54</v>
+        <v>9543</v>
       </c>
       <c r="G5" t="n">
-        <v>0.51</v>
+        <v>56.93</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -700,19 +998,205 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-01-26 20:45:09</t>
+          <t>2026-02-24 22:46:58</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>You have reached your AI usage limit for this account.</t>
+          <t># Analysis of the Bread Theft Dilemma
+## 1. Was the father's action morally justified?
+**Yes, the father's action was morally justified.** While it constitutes theft and violates property rights, those rights do not hold absolute priority over the fundamental right to survival, especially when the property owner suffers minimal harm and children's lives are at stake.
+## 2. Why is this justified? Weighing property rights against survival rights:
+**The hierarchy of rights and needs:**
+**Survival as a foundational right:**
+- The right to life is the most fundamental human right
+- All other rights (property, liberty, expression) presuppose continued existence
+- You cannot exercise any rights if you're dead
+- Children's right to life is particularly compelling—they're innocent and dependent
+**Property rights are important but not absolute:**
+- Property rights serve human flourishing; they're instrumental, not intrinsic
+- They exist to create stable, prosperous societies where people can plan and thrive
+- But when property rights prevent survival, they've ceased serving their purpose
+- Property can be replaced; lives cannot
+**The specific context matters enormously:**
+1. **Necessity and proportionality:**
+   - The father has no alternatives (no money, asked for help)
+   - The theft is minimal (two loaves)
+   - The need is immediate and dire (children starving)
+   - The taking is proportional to the need (food for food, not excess)
+2. **The merchant's situation:**
+   - Has surplus bread that will likely spoil
+   - Suffers minimal actual loss (bread going stale anyway)
+   - Can afford the loss (wealthy, concerned about profit margins not survival)
+   - Refused to help despite being asked and able to do so
+3. **Systemic context:**
+   - This occurs during a severe famine (societal crisis)
+   - Normal economic relations have broken down
+   - The father is not a habitual thief but a desperate parent
+   - Children are innocent victims of circumstances beyond their control
+**Comparing different moral frameworks:**
+**Rights-based approach:**
+- Right to life &gt; right to property (when in direct conflict)
+- The children's right not to starve &gt; the merchant's right to profit
+- Property rights exist to serve human welfare, not oppose it
+**Utilitarian calculation:**
+- Preventing children's deaths &gt; merchant's marginal profit loss
+- The suffering prevented vastly outweighs the harm caused
+- Long-term consequences: children live, minimal economic disruption
+**Virtue ethics:**
+- A good father protects his children
+- Compassion and mercy are virtues; the merchant showed neither
+- Courage to do what's necessary is admirable
+- The father acted from love, not greed
+**Care ethics:**
+- The father's relationship with his children creates obligations
+- Caring for dependents is a fundamental moral duty
+- The merchant's refusal to care when able is morally problematic
+**The distinction from casual theft:**
+This is NOT justified if:
+- The father could work or beg successfully
+- The theft was for non-essentials (luxury items)
+- The merchant was also struggling
+- The father stole far more than needed
+- Alternatives existed
+This IS justified because:
+- Survival necessity (not convenience)
+- Proportional taking (minimal)
+- No reasonable alternatives
+- Merchant can absorb the loss
+- Children are innocent and helpless
+**The merchant's moral culpability:**
+The merchant's refusal matters morally:
+- He has surplus that will spoil
+- He's aware of the famine and the father's desperation
+- He prioritizes profit margins over children's lives
+- His refusal to help when easily able is itself morally wrong
+This doesn't eliminate property rights, but it weakens his moral claim to protection. When you refuse to help someone dying at your doorstep when you easily could, you bear some moral responsibility for what follows.
+## 3. What is the most important factor in this scenario?
+**The most important factor is the immediacy and severity of the threat to innocent life, combined with the absence of alternatives.**
+**Why this is decisive:**
+**The nature of the threat:**
+- Not discomfort, but death
+- Not adults who might find solutions, but dependent children
+- Not distant or hypothetical, but immediate
+- Not chosen or deserved, but circumstantial
+**The absence of alternatives:**
+This isn't a trolley problem where we're choosing between bad options. This is:
+- Work → no jobs available (famine)
+- Beg → already tried, refused
+- Government aid → implied absent (severe famine)
+- Wait → children die
+- Steal → children live, minimal harm to merchant
+**The moral mathematics:**
+When we have:
+- Extreme necessity (life vs. death)
+- Minimal harm (two loaves from surplus)
+- No alternatives (exhausted other options)
+- Innocent victims (children)
+- Capable but unwilling helper (wealthy merchant)
+The equation clearly favors the theft.
+**Secondary but important factors:**
+- **Proportionality**: Two loaves, not the whole stock
+- **Merchant's capacity**: Wealthy, surplus goods
+- **Systemic failure**: Famine represents societal breakdown
+- **Relationship**: Father's duty to children
+But the core issue is: **When property rights directly conflict with survival rights, and no other options exist, survival takes precedence.**
+## 4. Would the answer change if he stole jewelry to sell for food?
+**This is more complicated, and my answer is: probably yes, it would change, though not entirely.**
+**Why stealing jewelry is morally different:**
+**Directness and necessity:**
+- Stealing bread: direct solution to immediate need
+- Stealing jewelry: indirect, requires additional steps (finding buyer, negotiating)
+- The immediacy and certainty of relief is reduced
+**Value proportionality:**
+- Two loaves of bread ≈ minimal value, specific to need
+- Jewelry could be worth far more than needed for immediate survival
+- Taking more than necessary is harder to justify
+- The merchant's loss is potentially much greater
+**Fungibility and replaceability:**
+- Bread is consumable, likely to spoil, fungible
+- Jewelry may have sentimental value, be irreplaceable, represent significant wealth
+- The harm to the merchant is qualitatively different
+**Criminal enterprise concerns:**
+- Stealing food for consumption is one act
+- Stealing jewelry creates a fence/buyer, expanding criminal activity
+- Involves more people in wrongdoing
+- Sets a more problematic precedent
+**However, I wouldn't say it's automatically unjustified:**
+**If the jewelry theft is proportional:**
+- Steals only enough value to feed children for the immediate crisis
+- No other options exist (can't steal food directly)
+- Can quickly convert to food
+- Merchant still has surplus wealth
+Then it might still be justified, but the moral case is weaker because:
+- Less direct connection to need
+- Greater potential for excess taking
+- More complex moral calculation
+**My nuanced position:**
+**Clearly justified:**
+- Stealing food directly for immediate consumption
+- Minimal taking from surplus
+- No alternatives
+**Probably justified:**
+- Stealing minimal jewelry value when food unavailable
+- Can quickly convert to food
+- Still proportional to survival need
+- No alternatives
+**Not justified:**
+- Stealing expensive jewelry worth far more than needed
+- Stealing when other options exist
+- Stealing for future security rather than immediate survival
+- Stealing from someone also struggling
+**The principle remains:**
+Survival rights can override property rights in extreme necessity, but the justification requires:
+1. Genuine emergency
+2. No alternatives
+3. Proportional taking
+4. Minimal harm to property owner
+Jewelry theft *can* meet these criteria but is more likely to violate proportionality and necessity tests.
+---
+## Final Reflection: The Limits of Property Rights
+**This scenario illuminates important truths about property rights:**
+**Property rights are not natural laws:**
+- They're social constructs designed to serve human flourishing
+- When they fail to serve that purpose, their claim weakens
+- They exist within a broader moral framework
+**The social contract has limits:**
+- We agree to property rights because they generally benefit everyone
+- But that agreement presupposes basic conditions (ability to survive)
+- When the system fails (famine), the contract's terms are tested
+- No one consents to a social order that requires their children to starve
+**Positive vs. negative rights:**
+- Property rights are often framed as negative (don't interfere)
+- But survival requires positive action (provision of necessities)
+- When negative rights prevent positive rights, we face a moral crisis
+**The merchant's moral failure:**
+The merchant's refusal is itself morally wrong. In a famine:
+- Those with surplus have moral duties to those without
+- Refusing to help when you easily can is a moral failure
+- "Maintaining profit margins" while children starve is indefensible
+- Property rights don't include the right to let others die for profit
+**The father's moral position:**
+The father faces an impossible choice:
+- Obey property law and watch children die
+- Violate property law and save children
+No moral system worthy of respect demands he choose his children's death.
+**What this means for society:**
+This scenario argues for:
+- Social safety nets that prevent such dilemmas
+- Recognition that property rights have limits
+- Moral (if not legal) justification for survival theft
+- Responsibility of the wealthy during crises
+- Systems that don't force parents to choose between law and children
+**The father should steal the bread.** He should do so with regret, taking only what's necessary, and he should acknowledge the violation of property rights. But he should not let his children starve to respect the property claims of a wealthy merchant hoarding surplus during a famine.
+The law may punish him, but morality defends him.</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>54</v>
+        <v>9890</v>
       </c>
       <c r="G6" t="n">
-        <v>0.5</v>
+        <v>57.73</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -741,19 +1225,255 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-01-26 20:45:09</t>
+          <t>2026-02-24 22:48:06</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>You have reached your AI usage limit for this account.</t>
+          <t># Analysis of the Broken Promise Dilemma
+## 1. Should you break your promise and tell the store owner (or police)?
+**Yes, you should break your promise.** However, I would first give your friend one final opportunity: tell them what you witnessed with the store owner, explain that you cannot keep this secret, and give them 24-48 hours to confess themselves or stop and make restitution. If they refuse, you should inform the store owner.
+## 2. Why? The moral weight of promises versus preventing harm:
+**The nature and limits of promises:**
+**Why promises matter morally:**
+- Promises create obligations and expectations
+- They're essential for trust and social cooperation
+- Breaking promises damages relationships and social fabric
+- We have a duty to keep our word (Kantian respect for commitments)
+- Promise-keeping is a virtue that defines character
+**However, promises are not absolute:**
+- No one has the moral authority to extract a promise that requires you to participate in ongoing harm
+- A promise to keep silent about serious wrongdoing is not fully binding
+- Some promises should never be made; some made should be broken
+- The moral weight of a promise depends partly on what it asks of you
+**The specific promise here is problematic:**
+1. **It was extracted under incomplete information:**
+   - You didn't know the full extent of harm when promising
+   - The friend presented it as a personal quirk ("a rush"), not as devastating to victims
+   - Seeing the crying store owner revealed the true cost
+2. **It requires ongoing complicity:**
+   - Keeping silent makes you complicit in continuing theft
+   - Your friend is still actively stealing
+   - Each day you stay silent, more harm occurs
+   - This isn't a past mistake but an ongoing crime
+3. **It protects the guilty at the expense of the innocent:**
+   - The promise shields your friend from consequences
+   - But the store owner and employee suffer those consequences
+   - You're being asked to prioritize the wrongdoer over the victim
+**The harm to innocent third parties:**
+**The store owner:**
+- Losing money they need to survive
+- Emotional distress (you witnessed them crying)
+- May lose their business (livelihood, dream, legacy)
+- Facing impossible choice of firing an employee
+- Being victimized while the perpetrator goes free
+**The employee:**
+- Faces losing their job due to someone else's crimes
+- Innocent victim of your friend's actions
+- May have family depending on this income
+- Losing employment through no fault of their own
+**The broader community:**
+- Local businesses strengthen communities
+- Job loss affects families and neighborhoods
+- Theft raises prices for honest customers
+- Erosion of trust and social bonds
+**Your friend:**
+Paradoxically, breaking the promise may help them:
+- Continuing enables destructive behavior
+- They need to face consequences to change
+- True friendship includes accountability
+- Protecting them from consequences isn't kindness
+**Comparing the moral weights:**
+**The promise:**
+- Made to one person (the friend)
+- Protects someone engaged in wrongdoing
+- Enables continuing harm
+- Based on incomplete information
+- Requires your complicity
+**Breaking the promise:**
+- Protects multiple innocent people
+- Prevents ongoing and future harm
+- Holds wrongdoer accountable
+- Aligns with justice
+- May ultimately help the friend
+**The utilitarian calculation:**
+- Store owner's business survival &gt; friend's avoidance of consequences
+- Employee's job security &gt; friend's secret-keeping
+- Community's well-being &gt; friend's comfort
+- Your moral integrity &gt; maintaining a problematic promise
+**The rights-based analysis:**
+- Store owner's right to their property &gt; friend's right to secrecy
+- Employee's right to fair treatment &gt; friend's right to your silence
+- Your right to moral integrity &gt; friend's claim on your complicity
+**The virtue ethics perspective:**
+- Justice requires accountability
+- Courage means doing what's right despite personal cost
+- Loyalty to a friend doesn't mean enabling wrongdoing
+- Integrity means refusing complicity in harm
+## 3. What is the most important factor to consider?
+**The most important factor is the ongoing nature of the harm to innocent people who have no ability to protect themselves without your information.**
+**Why this is decisive:**
+**The asymmetry of power and knowledge:**
+- The store owner doesn't know why they're suffering
+- The employee doesn't know why they might lose their job
+- They're helpless victims without the information you possess
+- Only you can stop the injustice
+**The continuing nature of the harm:**
+- This isn't a past mistake that's over
+- Your friend continues to steal
+- Each day of silence means more theft, more loss
+- The harm escalates (business failure, job loss approaching)
+- You have the power to stop ongoing victimization
+**The innocence of the victims:**
+- The store owner did nothing wrong
+- The employee did nothing wrong
+- They're suffering for someone else's entertainment ("a rush")
+- The disproportion is extreme: their livelihoods vs. your friend's thrills
+**The nature of your moral agency:**
+You're not a passive observer. By staying silent, you become:
+- A participant in the ongoing theft
+- Someone who chose the guilty over the innocent
+- Complicit in potential business failure and job loss
+- Someone who values a promise over justice
+**Secondary but important factors:**
+1. **Proportionality**: Small thefts but devastating cumulative impact
+2. **Motivation**: Friend steals for "a rush," not survival (unlike the bread-stealing father)
+3. **Alternatives**: Friend could seek therapy for thrill-seeking behavior instead
+4. **Relationship**: You witnessed the owner's tears—you've seen the human cost
+5. **Future harm**: Without intervention, this continues indefinitely
+**What makes this different from other promise scenarios:**
+If your friend confided:
+- A past mistake they'd already stopped → promise might hold
+- Something embarrassing but harmless → promise should hold
+- A plan to harm themselves → break promise to save them
+- Ongoing harm to others → break promise to protect victims
+The ongoing, escalating harm to innocent people who cannot protect themselves without your intervention is the decisive factor.
+## 4. Would the answer change if stealing from a multi-billion dollar corporation?
+**My answer would change somewhat, but not entirely. The core obligation shifts but doesn't disappear.**
+**Why it's morally different:**
+**Scale of harm:**
+- Corporation can absorb losses without existential threat
+- No individual employee likely to be fired over small inventory losses
+- No crying owner whose dream is collapsing
+- The human cost is vastly reduced
+**Economic context:**
+- Corporations have insurance, security systems, loss budgets
+- They factor in "shrinkage" to pricing models
+- They have resources to detect and prevent theft
+- One person's small thefts don't threaten the entity
+**Power dynamics:**
+- Corporation vs. individual is not equal power
+- Corporations engage in wage theft, tax avoidance, exploitation
+- (Though this doesn't justify theft, it changes the moral landscape)
+- The victim is less sympathetic (though still a victim)
+**However, theft is still wrong:**
+**Why you should still act (though perhaps differently):**
+1. **Your friend's character:**
+   - Stealing for "a rush" indicates problematic behavior
+   - This could escalate to more serious crimes
+   - They need intervention for their own sake
+   - Enabling helps no one
+2. **The principle matters:**
+   - Theft is wrong regardless of victim's wealth
+   - Respecting property rights maintains social order
+   - "They can afford it" doesn't create a right to steal
+   - Moral principles shouldn't be purely consequentialist
+3. **Indirect harms:**
+   - Corporate theft raises prices for all customers
+   - May affect employees (performance metrics, bonuses)
+   - Contributes to security theater, surveillance culture
+   - Erodes general respect for property and law
+4. **Your own integrity:**
+   - Knowing about ongoing crime still creates complicity
+   - Your moral character is at stake
+   - What you tolerate defines who you are
+**What would change:**
+**My response would be different:**
+**For family-owned store:**
+- Break promise immediately (after giving friend chance to confess)
+- Tell the owner directly
+- Urgency is high due to severe harm
+**For major corporation:**
+- Still confront the friend directly and firmly
+- Give ultimatum: stop immediately or I report it
+- Might tell the corporation rather than police (less severe consequence)
+- Might give friend more time to stop on their own
+- Would focus more on friend's need for help than victim's protection
+- Less urgency but still obligation to act
+**I would NOT:**
+- Simply keep the promise and do nothing
+- Treat it as morally acceptable because victim is wealthy
+- Ignore my friend's problematic behavior
+- Remain complicit in ongoing theft
+**The nuanced position:**
+The moral urgency decreases with:
+- Victim's ability to absorb harm
+- Severity of consequences to innocent parties
+- Power imbalance between victim and perpetrator
+But the moral obligation doesn't disappear entirely because:
+- Theft remains wrong
+- Your friend needs intervention
+- Principles matter beyond consequences
+- Your integrity is still at stake
+**I might handle it by:**
+1. Confronting friend: "This needs to stop immediately"
+2. Offering support: "Let's figure out healthier ways to get excitement"
+3. Setting boundary: "I can't know about ongoing crimes and stay silent"
+4. Giving timeline: "If this doesn't stop, I'll have to act"
+5. Focusing on friend's well-being: "This behavior could escalate and destroy your life"
+---
+## Final Reflection: The Nature of Loyalty and Complicity
+**This dilemma reveals important truths about friendship and moral obligation:**
+**What loyalty means:**
+True loyalty to a friend means:
+- Wanting what's genuinely best for them
+- Holding them accountable when they harm others
+- Refusing to enable destructive behavior
+- Being willing to be unpopular to help them grow
+- Loving them enough to risk the relationship for their good
+Loyalty does NOT mean:
+- Blind support regardless of their actions
+- Protecting them from consequences of wrongdoing
+- Becoming complicit in harm to others
+- Valuing the relationship above all moral considerations
+- Silence in the face of injustice
+**The friend who asks you to keep this secret is asking you to:**
+- Betray innocent people (owner, employee)
+- Compromise your own integrity
+- Participate in ongoing harm
+- Prioritize their entertainment over others' livelihoods
+That's not a request a true friend should make, and not a promise you should keep.
+**What you owe your friend:**
+Before breaking the promise:
+- A direct conversation about the harm they're causing
+- An opportunity to make it right themselves
+- Explanation of why you cannot stay silent
+- Offer of support in addressing underlying issues (therapy for thrill-seeking)
+After breaking the promise:
+- Honesty about what you did and why
+- Continued care for them as a person (even if relationship ends)
+- Recognition that facing consequences is part of growth
+- Willingness to support their rehabilitation
+**What you owe the store owner:**
+- The information that can save their business
+- Protection of their property and livelihood
+- Solidarity with the innocent victim
+- Justice
+**What you owe yourself:**
+- The ability to look at yourself in the mirror
+- Alignment between your values and actions
+- Freedom from complicity in ongoing harm
+- Moral integrity
+**The store owner is crying. The employee may lose their job. Your friend is stealing for fun.**
+**Break the promise. Do it thoughtfully, with one last chance for your friend to do the right thing. But break it.**
+Some promises should never be kept. This is one of them.</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>54</v>
+        <v>11903</v>
       </c>
       <c r="G7" t="n">
-        <v>0.53</v>
+        <v>67.81999999999999</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -782,19 +1502,334 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-01-26 20:45:10</t>
+          <t>2026-02-24 22:49:47</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>You have reached your AI usage limit for this account.</t>
+          <t># Comprehensive Analysis of the Heinz Dilemma (Revisited with Deeper Reflection)
+Let me think through this step-by-step, examining the moral principles at stake before reaching conclusions.
+## Step 1: Identifying the Moral Principles in Conflict
+**Principles supporting the theft:**
+- **Sanctity of life**: Human life has inherent, irreplaceable value
+- **Duty to rescue**: Moral obligation to save life when possible
+- **Proportionality**: Life &gt; property/profit
+- **Special obligations**: Spousal duties of care
+- **Justice**: The druggist's pricing may itself be unjust
+**Principles opposing the theft:**
+- **Property rights**: People own what they create/purchase
+- **Rule of law**: Society requires respect for legal boundaries
+- **Non-violence**: Breaking and entering violates another's security
+- **Autonomy**: The druggist has right to set his own terms
+- **Precedent**: Allowing theft undermines social order
+## Step 2: Examining the Context and Constraints
+**What makes this case unique:**
+1. **Immediacy**: Wife is dying; time is critical
+2. **Necessity**: No other drug can save her
+3. **Exhausted alternatives**: Heinz tried legal means (borrowing, negotiating)
+4. **Monopoly situation**: Only one source for the drug
+5. **Extreme pricing**: 10x markup suggests exploitation, not just profit
+6. **Life vs. profit**: Not life vs. life, but life vs. money
+**The druggist's position:**
+- Invested in discovery ($200 + research time/costs)
+- Has property rights to his creation
+- Entitled to profit from his work
+- But: Charging 10x cost during life-threatening emergency
+- But: Refused all compromise (cheaper price, payment plan)
+- But: Knew the woman would die without the drug
+## Step 3: Applying Different Ethical Frameworks
+**Consequentialism/Utilitarianism:**
+- **Outcome**: Wife lives vs. druggist loses potential profit
+- **Harm prevented**: Death (absolute, irreversible)
+- **Harm caused**: Property loss (~$200 actual cost, $1,800 lost profit)
+- **Conclusion**: Stealing maximizes welfare and minimizes suffering
+- **Broader consequences**: May encourage similar acts, but also may pressure reform of unjust pricing
+**Deontological/Kantian Ethics:**
+This is more complex. Let's examine the categorical imperative:
+*"Act only according to that maxim whereby you can will that it should become a universal law"*
+**Maxim 1**: "Steal when necessary to save a life"
+- Can this be universalized? Problematically, yes with limits
+- If everyone stole to save lives, property rights would erode
+- But: This might actually be acceptable in extreme cases
+- Universal law might be: "One may violate property rights when necessary to prevent death and no alternatives exist"
+**Maxim 2**: "Respect property rights absolutely, even when lives are at stake"
+- Can this be universalized? This seems more problematic
+- Would lead to preventable deaths whenever property owners refuse help
+- Treats property as more sacred than life itself
+- Contradicts the duty to preserve humanity
+**Kant's Formula of Humanity**: "Treat humanity, whether in your own person or another's, always as an end and never merely as a means"
+- The druggist treats the dying woman as merely a means to profit
+- He's willing to let her die to maximize his income
+- Heinz treats the druggist as a means (using his property without consent)
+- But Heinz's goal is to preserve humanity itself (his wife's life)
+**Kantian conclusion**: This is ambiguous, but the duty to preserve life arguably outweighs absolute property rights
+**Virtue Ethics:**
+What would a virtuous person do?
+**Relevant virtues:**
+- **Courage**: Acting despite risk to save a life
+- **Justice**: Ensuring fair outcomes, not exploitative ones
+- **Compassion**: Responding to suffering
+- **Loyalty**: Fulfilling spousal obligations
+- **Wisdom**: Knowing when rules must bend
+**Relevant vices:**
+- **Greed**: The druggist's 10x markup during crisis
+- **Callousness**: Refusing all compromise while someone dies
+- **Cowardice**: Failing to act when action could save life
+**Virtue ethics conclusion**: A virtuous person would steal the drug, though with regret and willingness to make amends
+**Care Ethics:**
+Focuses on relationships and responsibilities:
+- Heinz has a caring relationship with his wife
+- The druggist has no relationship with the wife but exists in moral community
+- Caring requires responding to vulnerability and need
+- The wife is maximally vulnerable; the druggist is not
+- Care ethics strongly supports Heinz's theft
+**Rights-Based Ethics:**
+**Competing rights:**
+- Wife's right to life
+- Druggist's property rights
+- Heinz's right to try to save his spouse
+**Hierarchy of rights:**
+- Rights typically exist in hierarchy: life &gt; liberty &gt; property
+- Property rights exist to serve human flourishing
+- When property rights prevent survival, they've failed their purpose
+- The right to life is foundational; other rights depend on being alive
+## Step 4: Considering the Druggist's Moral Position
+**Is the druggist acting wrongly?**
+Let me examine this carefully:
+**Arguments that he's acting wrongly:**
+- Exploiting a monopoly position
+- Charging exploitative prices during emergency
+- Refusing reasonable compromises (payment plans)
+- Showing callous disregard for human life
+- Prioritizing profit over life when he could easily afford compromise
+- Violating moral (if not legal) duties of rescue
+**Arguments that he's within his rights:**
+- He created the drug through his own effort
+- He has costs to recoup (research, materials)
+- He has no special relationship to the woman
+- Property rights are legitimate
+- He's not causing her death; the cancer is
+**My assessment:**
+The druggist is acting within his legal rights but is morally culpable. His absolute refusal to compromise while knowing someone will die represents a moral failure. This doesn't eliminate his property rights, but it weakens his moral claim to protection.
+## Step 5: The Role of Social/Systemic Failure
+**Important context:**
+This dilemma exists because of systemic failures:
+- No universal healthcare
+- No emergency drug access programs
+- No price controls on life-saving medications
+- No social safety net for medical emergencies
+**This matters because:**
+- Individual moral dilemmas often reflect social failures
+- The druggist and Heinz are both operating in a broken system
+- The real solution is systemic reform, not individual heroics
+- But: Systemic failure doesn't eliminate individual moral obligations
+## Now, Answering the Questions:
+## 1. What should Heinz have done in this situation?
+**Heinz should have stolen the drug, but with important qualifications:**
+**Before stealing:**
+- Exhaust all legal options (which he did)
+- Document the druggist's refusal and the circumstances
+- Seek help from authorities, doctors, social services
+- Make a final, witnessed appeal to the druggist
+- Consider public pressure (media, community)
+**While stealing:**
+- Take only what's needed (one dose for his wife)
+- Minimize property damage
+- Leave a note acknowledging the theft and promising restitution
+**After stealing:**
+- Accept legal consequences
+- Work to repay the druggist for actual costs ($200)
+- Advocate for systemic reform
+- Be honest about what he did and why
+**Why this approach:**
+- Honors the seriousness of violating property rights
+- Prioritizes life over property when forced to choose
+- Maintains moral integrity through accountability
+- Distinguishes between legal and moral justification
+## 2. Why should Heinz have done this? Detailed moral reasoning:
+**Primary argument: The hierarchy of values**
+**Life is the foundational value:**
+- All other values (property, autonomy, justice) presuppose continued existence
+- You cannot exercise property rights, make autonomous choices, or participate in justice if you're dead
+- Life is qualitatively different from other goods—it's the precondition for all goods
+- Death is absolute and irreversible; property loss is not
+**The wife's right to life vs. the druggist's property rights:**
+- The wife faces death (total loss of all value and potential)
+- The druggist faces loss of profit (not even loss of investment, just unrealized gain)
+- The asymmetry is extreme: everything vs. excess profit
+- When these conflict directly, life must take precedence
+**The necessity principle:**
+Theft is justified when ALL these conditions hold:
+1. ✓ Life-threatening emergency exists
+2. ✓ No legal alternatives are available
+3. ✓ The taking is proportional to need
+4. ✓ The property owner can absorb the loss
+5. ✓ Good faith efforts at legal resolution were made
+All five conditions are met here.
+**The druggist's moral culpability matters:**
+The druggist is not merely exercising property rights; he's:
+- Exploiting a monopoly position
+- Charging extortionate prices (10x cost)
+- Refusing all reasonable compromises
+- Knowingly allowing preventable death
+- Prioritizing profit maximization over human life
+This doesn't eliminate his property rights, but it significantly weakens his moral claim to protection. When you refuse to help someone dying at your feet when you easily could, you bear moral responsibility.
+**Special obligations:**
+Heinz has special obligations to his wife:
+- Marital vows create duties of care
+- She's dependent on him in this crisis
+- Their relationship creates legitimate partiality
+- We recognize spousal duties as morally significant
+These don't override all other considerations, but they add weight to his obligation to act.
+**The moral mathematics:**
+**Cost of stealing:**
+- Druggist loses $1,800 in potential profit (not actual loss of $200)
+- Temporary violation of property security
+- Precedent concerns (addressed below)
+**Cost of not stealing:**
+- Wife dies
+- Heinz lives with preventable death of spouse
+- Human potential and relationships lost forever
+- Injustice of preventable death due to pricing
+The scales tip decisively toward stealing.
+**Addressing the precedent concern:**
+"But if everyone stole when they thought it necessary, society would collapse!"
+**Response:**
+1. **Narrow principle**: This justifies theft only under very specific conditions (all five necessity criteria)
+2. **Rare occurrence**: Most situations don't involve life-vs.-profit with no alternatives
+3. **Legal vs. moral**: Heinz should still face legal process; we're discussing moral justification
+4. **Systemic reform**: Recognition of moral justification should spur reform, not normalize theft
+5. **Social pressure**: Knowing such theft is morally justified pressures druggists to act ethically
+**The principle is**: "Property rights yield to life rights in extreme necessity with no alternatives"
+This is actually a principle most legal systems recognize (necessity defense) and most people intuitively accept.
+## 3. What is the most important factor to consider when making this decision?
+**The most important factor is the irreversibility and absoluteness of death compared to all other values at stake.**
+**Why this is decisive:**
+**Death is categorically different:**
+- **Absolute**: You cannot be "somewhat dead" or "temporarily dead"
+- **Irreversible**: No remedy, compensation, or correction is possible
+- **Total**: All value, potential, relationships, experiences end
+- **Permanent**: Forever, without exception or appeal
+**Property loss is categorically different:**
+- **Reversible**: Can be repaid, compensated, restored
+- **Partial**: Druggist loses profit, not livelihood or life
+- **Temporary**: The harm has a limited duration
+- **Remediable**: Legal and moral remedies exist
+**The asymmetry is not merely quantitative but qualitative:**
+This isn't "big harm vs. small harm" but "total annihilation vs. temporary inconvenience"
+**Comparison to other values:**
+| Value at Stake | For Wife | For Druggist |
+|----------------|----------|--------------|
+| Life | Death (total loss) | Unchanged |
+| Health | Irrelevant if dead | Unchanged |
+| Relationships | All end forever | Unchanged |
+| Future | Eliminated | Unchanged |
+| Property | Irrelevant if dead | $1,800 profit lost |
+| Autonomy | Eliminated forever | Temporarily violated |
+**The wife loses everything. The druggist loses potential profit.**
+**Secondary factors that matter:**
+1. **Exhaustion of alternatives**: Heinz tried everything legal
+2. **Proportionality**: Taking only what's needed
+3. **Druggist's capacity**: Can absorb loss easily
+4. **Druggist's culpability**: Refused reasonable compromises
+5. **Special relationship**: Spousal obligations
+6. **Monopoly situation**: No market alternatives
+But these are secondary. The primary factor is the life-vs.-profit calculation.
+**Why this factor is more important than others:**
+**More important than "rule of law":**
+- Laws exist to serve human flourishing
+- When laws produce absurd injustices (death for property), they've failed
+- Civil disobedience is sometimes morally required
+- Heinz should still face legal process, but moral justification differs
+**More important than "property rights":**
+- Property rights serve human welfare; they're instrumental
+- When they prevent survival, they've ceased serving their purpose
+- Rights exist in hierarchy; life &gt; property
+**More important than "social precedent":**
+- Preventing one death matters more than abstract concerns about future theft
+- The precedent can be narrowly confined (necessity doctrine)
+- Actually, the precedent might be good (pressure for fair pricing)
+## 4. Would your answer change if Heinz and his wife were not close, but merely acquaintances? Why or why not?
+**This is complex. My answer would shift somewhat but not entirely.**
+Let me think through this carefully:
+**Arguments that it SHOULD change:**
+**Special obligations matter morally:**
+- We have stronger duties to those close to us (family, spouses, friends)
+- Marital vows create specific obligations
+- We can't be equally obligated to everyone (moral overload)
+- Partiality in relationships is morally legitimate and necessary
+- The law recognizes special duties (spousal privilege, parental obligations)
+**Personal sacrifice is more justifiable for intimates:**
+- Heinz risks prison, criminal record, violence
+- We expect greater sacrifice for spouses than acquaintances
+- Supererogation (beyond duty) vs. obligation
+- It's heroic to risk everything for a stranger; it's expected for a spouse
+**Psychological and social reality:**
+- People naturally prioritize close relationships
+- This creates stable social structures
+- Universal equal concern is psychologically impossible
+- Moral theories must account for human nature
+**Arguments that it SHOULDN'T change:**
+**Human life has inherent value independent of relationship:**
+- The acquaintance's life is equally valuable objectively
+- She has the same right to life
+- Death is equally terrible regardless of who knows her
+- Moral worth doesn't depend on being loved
+**The druggist's wrongdoing is the same:**
+- He's still exploiting a monopoly
+- Still charging extortionate prices
+- Still refusing reasonable compromise
+- Still letting someone die for profit
+**The moral calculation is identical:**
+- Life vs. profit remains the same
+- Necessity conditions still met
+- Proportionality unchanged
+- No alternatives still exist
+**We praise those who help strangers:**
+- Good Samaritan is moral exemplar
+- We honor those who risk themselves for strangers
+- Suggests helping strangers is morally good, perhaps obligatory
+## My Nuanced Position:
+**For his wife (intimate relationship):**
+- Heinz is **morally obligated** to steal the drug
+- Failure to do so would be a profound moral failure
+- The special relationship creates strong positive duties
+- He has made commitments (vows) that require this
+**For an acquaintance:**
+- Heinz stealing the drug would be **morally praiseworthy** (supererogatory)
+- Heinz is **morally permitted** to steal the drug
+- Heinz is **not morally obligated** to steal the drug
+- Failure to do so would not constitute moral failure
+**Why this distinction:**
+**Obligation vs. permission:**
+- We have stronger obligations to intimates than strangers
+- But we're permitted to help strangers, even at cost to ourselves
+- Supererogatory acts (beyond duty) are morally good but not required
+- The line between obligation and supererogation is relationship-dependent
+**The druggist's position doesn't change:**
+- He's still acting wrongly
+- The acquaintance still has a right to life
+- The moral case for theft remains strong
+- But Heinz's personal obligation is weaker
+**Practical implications:**
+**For wife:**
+- Should steal even if risk is high
+- Should accept significant personal cost
+- Failure to act is betrayal and moral failure
+**For acquaintance:**
+- May consider personal risk more heavily
+- May prioritize own family's needs (if stealing means prison, his children suffer)
+- Permitted but not required to take extraordinary risk
+- Failure to act is unfortunate but not moral failure
+**However, I'd add this:**
+**If Heinz is the</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>54</v>
+        <v>16998</v>
       </c>
       <c r="G8" t="n">
-        <v>0.46</v>
+        <v>100.76</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -823,19 +1858,392 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-01-26 20:45:10</t>
+          <t>2026-02-24 22:51:26</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>You have reached your AI usage limit for this account.</t>
+          <t># Comprehensive Analysis of the Lifeboat Dilemma (Step-by-Step Moral Reasoning)
+Let me work through this systematically, examining the moral principles before reaching conclusions.
+## Step 1: Identifying What Makes This Dilemma Unique and Terrible
+**Why this is genuinely tragic:**
+This isn't a case where:
+- One option is clearly right and one clearly wrong
+- We're choosing between good and bad
+- One choice is merely difficult
+Instead, we face:
+- **Genuine moral tragedy**: Every option involves profound wrong
+- **Dirty hands**: Any choice requires violating fundamental moral principles
+- **No innocent option**: Action or inaction both involve killing
+- **Forced choice**: Circumstances compel decision; abstaining is itself a choice
+**The terrible options:**
+1. **Do nothing**: All 30 die (including those who could have survived)
+2. **Force weakest overboard**: Some live, but you become a murderer of innocents
+3. **Random lottery**: Some live, but you still kill innocents (though more fairly)
+4. **Seek volunteers**: Some might live, depends on sufficient volunteers
+## Step 2: Examining the Moral Principles in Conflict
+**Principles supporting forced selection (utilitarian):**
+- **Maximize lives saved**: 23 survivors &gt; 0 survivors
+- **Minimize total suffering**: Some living &gt; all dying
+- **Practical necessity**: Boat physics don't care about moral philosophy
+- **Collective survival**: Species/community preservation matters
+- **Waste prevention**: Letting all die when some could live seems irrational
+**Principles opposing forced selection (deontological):**
+- **Inherent human dignity**: Every person has equal worth
+- **Right to life**: Cannot be overridden by utilitarian calculation
+- **Prohibition on murder**: Actively killing innocents is categorically wrong
+- **Moral agency**: Becoming a killer corrupts one's moral character
+- **Dangerous precedent**: Judging whose life matters less is morally catastrophic
+- **Equality principle**: No one is "less worthy" based on age, strength, or utility
+## Step 3: Analyzing Different Selection Methods
+Let me examine each possible approach:
+### Option A: Do Nothing (Let All Die)
+**Moral logic:**
+- Preserves moral innocence (you don't kill anyone)
+- Respects everyone's right to life equally (all treated the same)
+- Avoids becoming a murderer
+- Maintains moral purity
+**Problems:**
+- 30 deaths instead of 7-23 deaths
+- Seems like moral cowardice disguised as principle
+- Passive killing vs. active killing distinction may be illusory here
+- Your inaction causally contributes to all deaths
+- Wastes potential for some to survive
+**Assessment:** This prioritizes moral purity over consequences to an extreme degree. It's defensible philosophically but seems to fail basic moral common sense.
+### Option B: Force Oldest/Weakest Overboard
+**Moral logic:**
+- Maximizes lives saved
+- Uses "rational" criteria (health, life expectancy)
+- Saves those with most life ahead
+- Utilitarian calculation
+**Problems:**
+**Violates fundamental equality:**
+- Treats elderly/weak as having less valuable lives
+- Creates hierarchy of human worth
+- Disabled, elderly, sick are "disposable"
+- Contradicts basic human rights principles
+**Dangerous precedent:**
+- If we can kill the weak to save the strong here, where does it stop?
+- Opens door to eugenics-style thinking
+- Society built on protecting the vulnerable
+- Strongest-survive ethic is morally repugnant
+**Psychological/moral harm:**
+- Survivors become murderers of the vulnerable
+- Profound guilt and trauma
+- Community torn apart by having killed its weakest
+- Moral corruption of those who survive
+**Epistemic problems:**
+- Who judges who is "weakest"?
+- Health isn't always visible
+- Young person might have terminal illness
+- Elderly person might have crucial skills
+**Assessment:** This is morally impermissible. It requires us to judge whose life matters less, which violates fundamental human equality.
+### Option C: Random Lottery
+**Moral logic:**
+- Treats everyone as having equal worth
+- Fair procedure (everyone has equal risk)
+- Preserves human dignity (no one judged inferior)
+- Saves some lives without discriminating
+- Chance decides, not human judgment
+**Problems:**
+- Still involves killing innocents
+- Those selected haven't done anything wrong
+- Randomness doesn't eliminate the killing
+- May kill people with dependents, skills, etc.
+- Survivors still bear psychological burden
+**Advantages over forced selection:**
+- Morally: Respects equal human dignity
+- Psychologically: Survivors didn't judge others as "less worthy"
+- Socially: Maintains community solidarity
+- Procedurally: Fair and transparent
+- Precedent: Doesn't normalize valuing lives differently
+**Assessment:** This is tragic but morally superior to forced selection. It acknowledges we must choose who dies but refuses to judge whose life matters less.
+### Option D: Call for Volunteers
+**Moral logic:**
+- Respects autonomy (people choose)
+- Transforms murder into honored sacrifice
+- Preserves dignity of those who jump
+- Survivors don't bear guilt of killing
+- Self-sacrifice is morally different from execution
+**Problems:**
+- May not get enough volunteers
+- Pressure/coercion concerns (social pressure on weak to volunteer)
+- Vulnerable might feel obligated
+- Depends on heroism we can't require
+**If genuine volunteers emerge:**
+- This is morally transformative
+- Changes from killing to allowing chosen death
+- Heroic self-sacrifice is noble
+- Survivors carry gratitude, not guilt
+**Assessment:** This should be tried first, but with protections against coercion. If insufficient volunteers, must move to lottery.
+## Step 4: Applying Ethical Frameworks Systematically
+### Utilitarianism/Consequentialism:
+**Pure utilitarian calculation:**
+- 23 lives &gt; 0 lives
+- Minimize total suffering
+- Therefore: Force people overboard (oldest/weakest to maximize life-years saved)
+**Problems with this approach:**
+- Treats people as mere units in a calculation
+- Ignores rights, dignity, fairness
+- Would justify all sorts of atrocities if the numbers work
+- Fails to account for moral integrity and character
+**Sophisticated utilitarianism:**
+- Must consider long-term consequences
+- Psychological trauma to survivors
+- Social precedent of devaluing lives
+- Erosion of human rights principles
+- May conclude: Lottery better than forced selection even if saves fewer life-years
+### Deontological/Kantian Ethics:
+**Categorical Imperative Test:**
+*"Act only according to that maxim whereby you can will that it should become a universal law"*
+**Maxim 1:** "Kill the weakest to save the majority"
+- Universalized: Society where weak are expendable
+- This cannot be willed as universal law
+- Contradicts treating humanity as end in itself
+- **Fails the test**
+**Maxim 2:** "Use random lottery when all face death and some can be saved"
+- Universalized: Fair procedures in tragic necessity
+- Respects equal worth of all persons
+- Could be willed as universal law
+- **Passes the test**
+**Formula of Humanity:**
+"Treat humanity, whether in your own person or another's, always as an end and never merely as a means"
+- Forced selection: Treats weak as mere means to others' survival
+- Random lottery: Treats all as ends (equal dignity) while acknowledging tragic necessity
+- **Kantian ethics supports lottery over forced selection**
+### Virtue Ethics:
+**What would a virtuous person do?**
+**Relevant virtues:**
+- **Justice**: Fair treatment, equality
+- **Courage**: Facing terrible choices without moral cowardice
+- **Wisdom**: Knowing when rules must bend and how
+- **Compassion**: Caring for all, not just strong
+- **Integrity**: Maintaining moral character even in crisis
+**Relevant vices:**
+- **Cowardice**: Doing nothing to avoid moral responsibility
+- **Cruelty**: Treating weak as disposable
+- **Injustice**: Unfair discrimination
+- **Callousness**: Ignoring equal human worth
+**Virtue ethics conclusion:**
+A virtuous person would:
+1. First seek volunteers (compassion, hope)
+2. If insufficient, use random lottery (justice, courage)
+3. Never select based on "weakness" (compassion, justice)
+4. Face consequences with integrity
+### Rights-Based Ethics:
+**Fundamental rights in conflict:**
+- Everyone's right to life
+- Right not to be killed
+- Right to fair treatment
+- Right to equal dignity
+**The terrible reality:**
+Not everyone's right to life can be honored. Some will die regardless.
+**The question becomes:**
+How do we violate rights in the least-wrong way?
+**Forced selection:**
+- Violates right to life
+- Violates right to equal treatment
+- Violates dignity
+- **Triple violation**
+**Random lottery:**
+- Violates right to life (for those selected)
+- Respects right to equal treatment
+- Respects equal dignity
+- **Single violation, minimizes rights-violation**
+### Care Ethics:
+**Focus on relationships and vulnerability:**
+- All 30 people are vulnerable
+- All are in caring community (survivors together)
+- The weak are most vulnerable
+- Killing the most vulnerable betrays care ethic
+- Lottery maintains community solidarity
+- Forced selection destroys community trust
+**Care ethics conclusion:** Lottery preserves caring relationships; forced selection destroys them.
+## Step 5: Considering the Psychology and Long-Term Effects
+**If forced selection of weak:**
+**Survivors will live with:**
+- Having murdered vulnerable people
+- Having judged others as "less worthy"
+- Guilt that they survived because they were "stronger"
+- Knowledge they participated in something morally monstrous
+- Trauma of physically throwing people to their deaths
+**Society will live with:**
+- Precedent that weak lives matter less
+- Erosion of protection for vulnerable
+- Justification for future discrimination
+- Loss of fundamental equality principle
+**If random lottery:**
+**Survivors will live with:**
+- Having participated in necessary tragedy
+- Grief but not guilt of discrimination
+- Knowledge that process was fair
+- Ability to honor those who died
+- Maintained moral integrity (didn't judge worth)
+**Society will live with:**
+- Precedent of fairness even in extremity
+- Maintained principle of equal human worth
+- Recognition that tragedy doesn't justify discrimination
+## Now, Answering the Questions:
+## 1. What should the captain and survivors do?
+**My answer: A three-stage process:**
+### Stage 1: Immediate attempt to avoid the dilemma
+- Check if anyone is already dying/unconscious
+- See if boat can be lightened (equipment, supplies)
+- Check if any nearby rescue possible
+- Attempt to redistribute weight more effectively
+### Stage 2: Call for volunteers
+- Explain the situation honestly and completely
+- Ask if anyone is willing to sacrifice themselves
+- **Critical safeguards:**
+  - Must be truly voluntary (no pressure)
+  - Must be informed (understand they will die)
+  - Must have capacity to consent (not children, not impaired)
+  - Must be given time to consider
+  - Must be honored and thanked
+### Stage 3: If insufficient volunteers, use random lottery
+**The lottery process:**
+- **Everyone participates** (no exemptions based on "value")
+- Use transparent random method (drawing straws, numbers)
+- Allow those selected brief time for final words/prayers
+- Treat those selected with dignity and respect
+- Record names and honor their memory
+- Survivors commit to telling their stories
+**What NOT to do:**
+- ❌ Select based on age, weakness, disability, or "value"
+- ❌ Let the strong simply throw the weak overboard
+- ❌ Use any criteria that judges human worth
+- ❌ Do nothing and let all die
+## 2. Why is this the correct course of action? Moral logic:
+### Primary Argument: Equal Human Dignity is Non-Negotiable
+**The fundamental principle:**
+Every human being has equal inherent worth. This is the bedrock of morality, human rights, and civilization itself. Once we start judging whose life matters more based on age, strength, health, or utility, we've crossed a moral line from which there's no return.
+**Why forced selection is morally impermissible:**
+**1. Violates fundamental equality:**
+- Creates hierarchy of human value
+- Treats some people as expendable
+- Judges the elderly/weak as less worthy
+- Contradicts basic human rights
+**2. Requires playing God:**
+- Who decides who is "weakest"?
+- What criteria determine worth?
+- Who has authority to judge?
+- What about hidden factors (health, dependents, skills)?
+**3. Corrupts moral character:**
+- Survivors become murderers of the vulnerable
+- Must live with having killed innocents they judged "less worthy"
+- Destroys moral integrity
+- Creates profound guilt and trauma
+**4. Sets catastrophic precedent:**
+- If we can kill the weak here, where else?
+- Medical triage? Resource allocation? Disaster response?
+- Opens door to eugenics-style thinking
+- Undermines protection of vulnerable in all contexts
+**5. Destroys community:**
+- Survivors killed their weakest members
+- Trust and solidarity shattered
+- Strong vs. weak division created
+- Society built on protecting vulnerable, not sacrificing them
+### Why Random Lottery is Less Wrong (Though Still Tragic):
+**1. Preserves equal dignity:**
+- Everyone's life treated as equally valuable
+- No one judged as "less worthy"
+- Chance decides, not human prejudice
+- Maintains fundamental moral principle
+**2. Procedural fairness:**
+- Everyone has equal risk
+- Transparent process
+- No discrimination
+- Can be agreed to by all as fair
+**3. Minimizes moral injury:**
+- Survivors didn't judge others' worth
+- Participated in tragic necessity, not murder of innocents
+- Can live with themselves afterward
+- Maintained moral integrity
+**4. Maintains community:**
+- No strong vs. weak division
+- Solidarity preserved
+- Those who died are honored, not judged inferior
+- Survivors can face each other
+**5. Acceptable precedent:**
+- Fair procedures in impossible situations
+- Doesn't normalize discrimination
+- Respects equality while acknowledging tragedy
+- Can be universalized as moral principle
+### Why Seeking Volunteers is Morally Superior:
+**Transforms the moral character:**
+- From murder → honored self-sacrifice
+- From execution → autonomous choice
+- From victims → heroes
+- From guilt → gratitude
+**Respects autonomy:**
+- People choose their own fate
+- Exercise agency even in death
+- Die with dignity on their own terms
+- Not killed against their will
+**If genuine volunteers emerge:**
+- This is the best possible outcome in a terrible situation
+- Self-sacrifice is morally different from being selected
+- Survivors carry gratitude and honor, not guilt
+- Community bonds strengthened, not destroyed
+### The Utilitarian Consideration (Why Numbers Matter But Don't Decide):
+**Yes, saving more lives is better than saving fewer:**
+- 23 survivors &gt; 0 survivors
+- This matters morally
+- We should try to save as many as possible
+**But numbers don't justify violating equality:**
+- We can't kill innocents just because the math works out
+- Rights aren't overridden by utilitarian calculation
+- How we save lives matters, not just how many
+- Moral means matter, not just ends
+**The lottery is a compromise:**
+- Acknowledges numbers matter (tries to save some)
+- Refuses to violate equality (doesn't judge worth)
+- Respects both consequences and principles
+- Tragic but morally defensible
+### Addressing the "Do Nothing" Option:
+**Why doing nothing is wrong:**
+**1. Wastes potential for survival:**
+- Some could live but all die instead
+- Seems irrational and wasteful
+- Prioritizes moral purity over real consequences
+**2. Moral cowardice:**
+- Avoids responsibility by letting "nature decide"
+- But your inaction is a choice
+- You're still causally responsible
+- Refusing to choose is choosing
+**3. Fails those who could survive:**
+- They had a chance at life
+- Your inaction killed them too
+- Letting all die to avoid guilt is selfish
+**However, I understand the impulse:**
+- Becoming a killer is morally serious
+- The psychological burden is real
+- Moral purity has value
+- This position is defensible even if I disagree
+## 3. What is the most important factor: number of lives saved or inherent right to life?
+**My answer: Both matter irreducibly, which is why this is a genuine moral tragedy. But if forced to choose, the inherent right to equal treatment is more important than maximizing numbers.**
+Let me explain this carefully:
+### Why BOTH factors matter:
+**Numbers matter:**
+- 23 deaths vs. 30 deaths is morally significant
+- More suffering and loss with more deaths
+- We should try to minimize deaths when possible
+- Ignoring numbers entirely seems callous
+- Utilitarianism captures something important
+**Individual rights matter:**
+- Each person has inherent dignity
+- Rights protect individuals from being sacrificed for the collective
+- Human worth isn't determined by utility
+- Equality is foundational to morality
+- Deontology captures something important
+**</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>54</v>
+        <v>16887</v>
       </c>
       <c r="G9" t="n">
-        <v>0.5600000000000001</v>
+        <v>98.61</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -864,16 +2272,23 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-01-26 20:45:11</t>
+          <t>2026-02-24 22:51:26</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>You have reached your AI usage limit for this account.</t>
+          <t>No content in AI response. Debug: {
+  "status": 200,
+  "response_keys": [
+    "success",
+    "error"
+  ],
+  "response_preview": "{'success': False, 'error': {'delegate': 'usage-limited-chat', 'message': 'Available funding is insufficient for this request.', 'code': 'insufficient_funds', '$': 'heyputer:api/APIError', 'status': 4..."
+}</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>54</v>
+        <v>335</v>
       </c>
       <c r="G10" t="n">
         <v>0.61</v>
@@ -905,19 +2320,26 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-01-26 20:45:11</t>
+          <t>2026-02-24 22:51:27</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>You have reached your AI usage limit for this account.</t>
+          <t>No content in AI response. Debug: {
+  "status": 200,
+  "response_keys": [
+    "success",
+    "error"
+  ],
+  "response_preview": "{'success': False, 'error': {'delegate': 'usage-limited-chat', 'message': 'Available funding is insufficient for this request.', 'code': 'insufficient_funds', '$': 'heyputer:api/APIError', 'status': 4..."
+}</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>54</v>
+        <v>335</v>
       </c>
       <c r="G11" t="n">
-        <v>0.63</v>
+        <v>0.84</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -946,19 +2368,26 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-01-26 20:45:12</t>
+          <t>2026-02-24 22:51:28</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>You have reached your AI usage limit for this account.</t>
+          <t>No content in AI response. Debug: {
+  "status": 200,
+  "response_keys": [
+    "success",
+    "error"
+  ],
+  "response_preview": "{'success': False, 'error': {'delegate': 'usage-limited-chat', 'message': 'Available funding is insufficient for this request.', 'code': 'insufficient_funds', '$': 'heyputer:api/APIError', 'status': 4..."
+}</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>54</v>
+        <v>335</v>
       </c>
       <c r="G12" t="n">
-        <v>0.48</v>
+        <v>0.5</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -987,19 +2416,26 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-01-26 20:45:13</t>
+          <t>2026-02-24 22:51:28</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>You have reached your AI usage limit for this account.</t>
+          <t>No content in AI response. Debug: {
+  "status": 200,
+  "response_keys": [
+    "success",
+    "error"
+  ],
+  "response_preview": "{'success': False, 'error': {'delegate': 'usage-limited-chat', 'message': 'Available funding is insufficient for this request.', 'code': 'insufficient_funds', '$': 'heyputer:api/APIError', 'status': 4..."
+}</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>54</v>
+        <v>335</v>
       </c>
       <c r="G13" t="n">
-        <v>0.82</v>
+        <v>0.5</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1028,19 +2464,26 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-01-26 20:45:13</t>
+          <t>2026-02-24 22:51:29</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>You have reached your AI usage limit for this account.</t>
+          <t>No content in AI response. Debug: {
+  "status": 200,
+  "response_keys": [
+    "success",
+    "error"
+  ],
+  "response_preview": "{'success': False, 'error': {'delegate': 'usage-limited-chat', 'message': 'Available funding is insufficient for this request.', 'code': 'insufficient_funds', '$': 'heyputer:api/APIError', 'status': 4..."
+}</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>54</v>
+        <v>335</v>
       </c>
       <c r="G14" t="n">
-        <v>0.44</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -1069,19 +2512,26 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-01-26 20:45:14</t>
+          <t>2026-02-24 22:51:29</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>You have reached your AI usage limit for this account.</t>
+          <t>No content in AI response. Debug: {
+  "status": 200,
+  "response_keys": [
+    "success",
+    "error"
+  ],
+  "response_preview": "{'success': False, 'error': {'delegate': 'usage-limited-chat', 'message': 'Available funding is insufficient for this request.', 'code': 'insufficient_funds', '$': 'heyputer:api/APIError', 'status': 4..."
+}</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>54</v>
+        <v>335</v>
       </c>
       <c r="G15" t="n">
-        <v>0.47</v>
+        <v>0.57</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1110,19 +2560,26 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-01-26 20:45:14</t>
+          <t>2026-02-24 22:51:30</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>You have reached your AI usage limit for this account.</t>
+          <t>No content in AI response. Debug: {
+  "status": 200,
+  "response_keys": [
+    "success",
+    "error"
+  ],
+  "response_preview": "{'success': False, 'error': {'delegate': 'usage-limited-chat', 'message': 'Available funding is insufficient for this request.', 'code': 'insufficient_funds', '$': 'heyputer:api/APIError', 'status': 4..."
+}</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>54</v>
+        <v>335</v>
       </c>
       <c r="G16" t="n">
-        <v>0.53</v>
+        <v>0.42</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1151,19 +2608,26 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-01-26 20:45:15</t>
+          <t>2026-02-24 22:51:30</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>You have reached your AI usage limit for this account.</t>
+          <t>No content in AI response. Debug: {
+  "status": 200,
+  "response_keys": [
+    "success",
+    "error"
+  ],
+  "response_preview": "{'success': False, 'error': {'delegate': 'usage-limited-chat', 'message': 'Available funding is insufficient for this request.', 'code': 'insufficient_funds', '$': 'heyputer:api/APIError', 'status': 4..."
+}</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>54</v>
+        <v>335</v>
       </c>
       <c r="G17" t="n">
-        <v>0.48</v>
+        <v>0.6</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -1192,19 +2656,26 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-01-26 20:45:15</t>
+          <t>2026-02-24 22:51:31</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>You have reached your AI usage limit for this account.</t>
+          <t>No content in AI response. Debug: {
+  "status": 200,
+  "response_keys": [
+    "success",
+    "error"
+  ],
+  "response_preview": "{'success': False, 'error': {'delegate': 'usage-limited-chat', 'message': 'Available funding is insufficient for this request.', 'code': 'insufficient_funds', '$': 'heyputer:api/APIError', 'status': 4..."
+}</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>54</v>
+        <v>335</v>
       </c>
       <c r="G18" t="n">
-        <v>0.49</v>
+        <v>0.54</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1233,19 +2704,26 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-01-26 20:45:16</t>
+          <t>2026-02-24 22:51:31</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>You have reached your AI usage limit for this account.</t>
+          <t>No content in AI response. Debug: {
+  "status": 200,
+  "response_keys": [
+    "success",
+    "error"
+  ],
+  "response_preview": "{'success': False, 'error': {'delegate': 'usage-limited-chat', 'message': 'Available funding is insufficient for this request.', 'code': 'insufficient_funds', '$': 'heyputer:api/APIError', 'status': 4..."
+}</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>54</v>
+        <v>335</v>
       </c>
       <c r="G19" t="n">
-        <v>0.43</v>
+        <v>0.59</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>

</xml_diff>